<commit_message>
chore(tracker): fila INFRA-01, migracion de compas a cluster propio (En curso)
P8 del PLAN-migracion-cluster.md: registrar la tarea antes de ejecutar
la Fase A. Sin fila previa para esta migracion en el tracker.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/COMPAS_Control_Desarrollo.xlsx
+++ b/docs/COMPAS_Control_Desarrollo.xlsx
@@ -924,7 +924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I192"/>
+  <dimension ref="A1:I193"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="12" min="1" max="1"/>
@@ -8786,6 +8786,48 @@
         </is>
       </c>
       <c r="I192" s="18" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>INFRA-01</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Migracion de COMPAS a cluster MongoDB propio (compas-prod, Atlas M0 us-east-1): dump del cluster viejo (sismo-v3), restore, switch de env vars en Render, verificacion y cierre documental. Ver PLAN-migracion-cluster.md</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Jorge + Sergio (Builders)</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Bitacora en docs/equipo/entregas/BUILD-migracion-cluster.md. Plan en docs/equipo/entregas/PLAN-migracion-cluster.md. Motivo: nodo enfermo en sismo-v3 cuelga el arranque del backend.</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>G1-G4</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I37"/>

</xml_diff>

<commit_message>
docs(tracker): registra hash del commit de cierre en INFRA-01
Completa la columna Evidencia de INFRA-01 con el hash del commit de
cierre de Fase D (a851305), que no podia autocitarse.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/COMPAS_Control_Desarrollo.xlsx
+++ b/docs/COMPAS_Control_Desarrollo.xlsx
@@ -8818,14 +8818,14 @@
           <t>Hecha</t>
         </is>
       </c>
-      <c r="G193" t="inlineStr">
+      <c r="G193" s="12" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
       <c r="H193" s="12" t="inlineStr">
         <is>
-          <t>Bitacora en docs/equipo/entregas/BUILD-migracion-cluster.md. Plan en docs/equipo/entregas/PLAN-migracion-cluster.md. Motivo: nodo enfermo en sismo-v3 cuelga el arranque del backend.</t>
+          <t>Bitacora en docs/equipo/entregas/BUILD-migracion-cluster.md. Plan en docs/equipo/entregas/PLAN-migracion-cluster.md. Motivo: nodo enfermo en sismo-v3 cuelga el arranque del backend. | Cierre: commit a851305 (docs/infra, Fase D)</t>
         </is>
       </c>
       <c r="I193" s="12" t="inlineStr">

</xml_diff>